<commit_message>
one quiz per page for demographic info
</commit_message>
<xml_diff>
--- a/demoquiz.xlsx
+++ b/demoquiz.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SPPA\CMKL\Animation_Project\Summer\Experiment_Workflows\Testing1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B32AE6-AA6E-491E-B3E2-C85A744F3F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A20200C-8CC9-453C-A42E-3FD7967EA171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="17472" windowHeight="10992" xr2:uid="{69E5977C-DF6D-4985-AA26-C707BB450112}"/>
   </bookViews>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>question</t>
   </si>
   <si>
-    <t>options</t>
-  </si>
-  <si>
     <t>What is your gender?</t>
   </si>
   <si>
@@ -56,19 +53,67 @@
     <t>What is your age?</t>
   </si>
   <si>
-    <t>Male|Female|Other|Prefer not to say</t>
-  </si>
-  <si>
-    <t>High school|Bachelor's degree|Master's degree|Doctoral degree</t>
-  </si>
-  <si>
-    <t>18-60</t>
-  </si>
-  <si>
-    <t>What is your English proficiency level?</t>
-  </si>
-  <si>
-    <t>A1 – Beginner |A2 – Elementary|B1 – Intermediate|B2 – Upper intermediate|C1 – Advanced|C2 – Proficient</t>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Prefer not to say</t>
+  </si>
+  <si>
+    <t>Bachelor's Degree</t>
+  </si>
+  <si>
+    <t>Master's Degree</t>
+  </si>
+  <si>
+    <t>Doctoral Degree</t>
+  </si>
+  <si>
+    <t>What is your English level?</t>
+  </si>
+  <si>
+    <t>High School</t>
+  </si>
+  <si>
+    <t>18 - 21</t>
+  </si>
+  <si>
+    <t>22 - 25</t>
+  </si>
+  <si>
+    <t>26 - 29</t>
+  </si>
+  <si>
+    <t>Over 29</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> I can only understand simple words and short sentences.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> I can understand most of the lecture well, though I might miss a few complex or technical terms.</t>
+  </si>
+  <si>
+    <t>I can effortlessly understand the entire lecture, including all advanced and technical terms.</t>
+  </si>
+  <si>
+    <t>I can understand basic sentences, but I cannot follow a continuous speech or lecture.</t>
   </si>
 </sst>
 </file>
@@ -443,54 +488,103 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1107768-35D9-46A5-ABEA-5C473E087043}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="31.47265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="90.15625" customWidth="1"/>
-    <col min="3" max="3" width="31.47265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="84.41796875" customWidth="1"/>
+    <col min="2" max="2" width="45.41796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="66.05078125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="75.7890625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="71.5234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>6</v>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="B16" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>